<commit_message>
test(fixtures): expand P4 sample to 20 rows for richer manual testing
Block A (10 rows): same email + same ASIN as a P3 order, with different
order_id / ship city / price / carrier. Produces 17 cross-shop product
repeats under `all:US`, including a pure cross-shop-only pair
(alice@ + A3 — singleton on each shop alone).

Block B (10 rows): same email as a P3 order but a NEW ASIN (A5–A8 are
P4-only). Each (buyer, asin) pair is unique across the whole dataset,
so these rows surface only in the buyer-history slide-over and do not
inflate the repeat-orders list.
</commit_message>
<xml_diff>
--- a/backend/tests/fixtures/sample_orders_p4.xlsx
+++ b/backend/tests/fixtures/sample_orders_p4.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X11"/>
+  <dimension ref="A1:X21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -550,7 +550,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>P4-O1</t>
+          <t>P4-A1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -599,16 +599,16 @@
         </is>
       </c>
       <c r="L2" s="1" t="n">
-        <v>45717.5</v>
+        <v>45718.5</v>
       </c>
       <c r="M2" s="1" t="n">
-        <v>45717.83333333334</v>
+        <v>45718.83333333334</v>
       </c>
       <c r="N2" s="1" t="n">
-        <v>45720.5</v>
+        <v>45721.5</v>
       </c>
       <c r="O2" t="n">
-        <v>9.99</v>
+        <v>11.99</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
@@ -620,7 +620,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -635,7 +635,7 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>TRK-P4-O1</t>
+          <t>TRK-P4-A1</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -658,42 +658,42 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>P4-O2</t>
+          <t>P4-A2</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>M-A2</t>
+          <t>M-A1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>K-A2</t>
+          <t>K-A1</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>S-GADGET</t>
+          <t>S-WIDGET</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Gadget A2</t>
+          <t>Widget A1</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Gadget</t>
+          <t>Widget</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Gadget A2 — single</t>
+          <t>Widget A1 — single</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -707,16 +707,16 @@
         </is>
       </c>
       <c r="L3" s="1" t="n">
-        <v>45725.5</v>
+        <v>45724.5</v>
       </c>
       <c r="M3" s="1" t="n">
-        <v>45725.83333333334</v>
+        <v>45724.83333333334</v>
       </c>
       <c r="N3" s="1" t="n">
-        <v>45728.5</v>
+        <v>45727.5</v>
       </c>
       <c r="O3" t="n">
-        <v>14.5</v>
+        <v>11.99</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
@@ -724,11 +724,11 @@
         </is>
       </c>
       <c r="Q3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>Dallas</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>TRK-P4-O2</t>
+          <t>TRK-P4-A2</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -766,42 +766,42 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>P4-O3</t>
+          <t>P4-A3</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>A4</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>M-A4</t>
+          <t>M-A1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>K-A4</t>
+          <t>K-A1</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>S-GIZMO</t>
+          <t>S-WIDGET</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Gizmo A4</t>
+          <t>Widget A1</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Gizmo</t>
+          <t>Widget</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Gizmo A4 — single</t>
+          <t>Widget A1 — single</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -815,16 +815,16 @@
         </is>
       </c>
       <c r="L4" s="1" t="n">
-        <v>45733.5</v>
+        <v>45731.5</v>
       </c>
       <c r="M4" s="1" t="n">
-        <v>45733.83333333334</v>
+        <v>45731.83333333334</v>
       </c>
       <c r="N4" s="1" t="n">
-        <v>45736.5</v>
+        <v>45734.5</v>
       </c>
       <c r="O4" t="n">
-        <v>24</v>
+        <v>11.99</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
@@ -836,7 +836,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -851,7 +851,7 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>TRK-P4-O3</t>
+          <t>TRK-P4-A3</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -874,42 +874,42 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>P4-O10</t>
+          <t>P4-A4</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>A2</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>M-A1</t>
+          <t>M-A2</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>K-A1</t>
+          <t>K-A2</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>S-WIDGET</t>
+          <t>S-GADGET</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Widget A1</t>
+          <t>Gadget A2</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Widget</t>
+          <t>Gadget</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Widget A1 — single</t>
+          <t>Gadget A2 — single</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -923,16 +923,16 @@
         </is>
       </c>
       <c r="L5" s="1" t="n">
-        <v>45767.5</v>
+        <v>45738.5</v>
       </c>
       <c r="M5" s="1" t="n">
-        <v>45767.83333333334</v>
+        <v>45738.83333333334</v>
       </c>
       <c r="N5" s="1" t="n">
-        <v>45770.5</v>
+        <v>45741.5</v>
       </c>
       <c r="O5" t="n">
-        <v>9.99</v>
+        <v>16.5</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
@@ -944,7 +944,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>Plano</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -959,12 +959,12 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>TRK-P4-O10</t>
+          <t>TRK-P4-A4</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>FedEx</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="W5" t="inlineStr"/>
@@ -982,42 +982,42 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>P4-O4</t>
+          <t>P4-A5</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>A2</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>M-A1</t>
+          <t>M-A2</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>K-A1</t>
+          <t>K-A2</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>S-WIDGET</t>
+          <t>S-GADGET</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Widget A1</t>
+          <t>Gadget A2</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Widget</t>
+          <t>Gadget</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Widget A1 — single</t>
+          <t>Gadget A2 — single</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -1027,20 +1027,20 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>frank@example.com</t>
+          <t>alice@example.com</t>
         </is>
       </c>
       <c r="L6" s="1" t="n">
-        <v>45722.5</v>
+        <v>45745.5</v>
       </c>
       <c r="M6" s="1" t="n">
-        <v>45722.83333333334</v>
+        <v>45745.83333333334</v>
       </c>
       <c r="N6" s="1" t="n">
-        <v>45725.5</v>
+        <v>45748.5</v>
       </c>
       <c r="O6" t="n">
-        <v>9.99</v>
+        <v>16.5</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
@@ -1052,12 +1052,12 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Fresno</t>
+          <t>Frisco</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1067,12 +1067,12 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>TRK-P4-O4</t>
+          <t>TRK-P4-A5</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>FedEx</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="W6" t="inlineStr"/>
@@ -1090,42 +1090,42 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>P4-O5</t>
+          <t>P4-A6</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>A3</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>M-A1</t>
+          <t>M-A3</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>K-A1</t>
+          <t>K-A3</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>S-WIDGET</t>
+          <t>S-DOO</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Widget A1</t>
+          <t>Doohickey A3</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Widget</t>
+          <t>Doohickey</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Widget A1 — single</t>
+          <t>Doohickey A3 — single</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1135,20 +1135,20 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>frank@example.com</t>
+          <t>alice@example.com</t>
         </is>
       </c>
       <c r="L7" s="1" t="n">
-        <v>45737.5</v>
+        <v>45752.5</v>
       </c>
       <c r="M7" s="1" t="n">
-        <v>45737.83333333334</v>
+        <v>45752.83333333334</v>
       </c>
       <c r="N7" s="1" t="n">
-        <v>45740.5</v>
+        <v>45755.5</v>
       </c>
       <c r="O7" t="n">
-        <v>9.99</v>
+        <v>22</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
@@ -1160,12 +1160,12 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Fresno</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>TRK-P4-O5</t>
+          <t>TRK-P4-A6</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
@@ -1198,42 +1198,42 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>P4-O6</t>
+          <t>P4-A7</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>M-A2</t>
+          <t>M-A1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>K-A2</t>
+          <t>K-A1</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>S-GADGET</t>
+          <t>S-WIDGET</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Gadget A2</t>
+          <t>Widget A1</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Gadget</t>
+          <t>Widget</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Gadget A2 — single</t>
+          <t>Widget A1 — single</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1243,20 +1243,20 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>greg@example.com</t>
+          <t>bob@example.com</t>
         </is>
       </c>
       <c r="L8" s="1" t="n">
-        <v>45729.5</v>
+        <v>45721.5</v>
       </c>
       <c r="M8" s="1" t="n">
-        <v>45729.83333333334</v>
+        <v>45721.83333333334</v>
       </c>
       <c r="N8" s="1" t="n">
-        <v>45732.5</v>
+        <v>45724.5</v>
       </c>
       <c r="O8" t="n">
-        <v>14.5</v>
+        <v>10.99</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
@@ -1268,12 +1268,12 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Gainesville</t>
+          <t>Cambridge</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1283,12 +1283,12 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>TRK-P4-O6</t>
+          <t>TRK-P4-A7</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>FedEx</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="W8" t="inlineStr"/>
@@ -1306,42 +1306,42 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>P4-O7</t>
+          <t>P4-A8</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>M-A2</t>
+          <t>M-A1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>K-A2</t>
+          <t>K-A1</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>S-GADGET</t>
+          <t>S-WIDGET</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Gadget A2</t>
+          <t>Widget A1</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Gadget</t>
+          <t>Widget</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Gadget A2 — single</t>
+          <t>Widget A1 — single</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1351,20 +1351,20 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>greg@example.com</t>
+          <t>bob@example.com</t>
         </is>
       </c>
       <c r="L9" s="1" t="n">
-        <v>45745.5</v>
+        <v>45735.5</v>
       </c>
       <c r="M9" s="1" t="n">
-        <v>45745.83333333334</v>
+        <v>45735.83333333334</v>
       </c>
       <c r="N9" s="1" t="n">
-        <v>45748.5</v>
+        <v>45738.5</v>
       </c>
       <c r="O9" t="n">
-        <v>14.5</v>
+        <v>10.99</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
@@ -1372,16 +1372,16 @@
         </is>
       </c>
       <c r="Q9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Gainesville</t>
+          <t>Worcester</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>FL</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -1391,7 +1391,7 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>TRK-P4-O7</t>
+          <t>TRK-P4-A8</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
@@ -1414,42 +1414,42 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>P4-O8</t>
+          <t>P4-A9</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>A2</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>M-A1</t>
+          <t>M-A2</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>K-A1</t>
+          <t>K-A2</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>S-WIDGET</t>
+          <t>S-GADGET</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Widget A1</t>
+          <t>Gadget A2</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Widget</t>
+          <t>Gadget</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Widget A1 — single</t>
+          <t>Gadget A2 — single</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1459,20 +1459,20 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>henry@example.com</t>
+          <t>dave@example.com</t>
         </is>
       </c>
       <c r="L10" s="1" t="n">
-        <v>45752.5</v>
+        <v>45727.5</v>
       </c>
       <c r="M10" s="1" t="n">
-        <v>45752.83333333334</v>
+        <v>45727.83333333334</v>
       </c>
       <c r="N10" s="1" t="n">
-        <v>45755.5</v>
+        <v>45730.5</v>
       </c>
       <c r="O10" t="n">
-        <v>9.99</v>
+        <v>15.99</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
@@ -1484,12 +1484,12 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Boulder</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>CO</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1499,7 +1499,7 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>TRK-P4-O8</t>
+          <t>TRK-P4-A9</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
@@ -1522,42 +1522,42 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>P4-O9</t>
+          <t>P4-A10</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>A4</t>
+          <t>A2</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>M-A4</t>
+          <t>M-A2</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>K-A4</t>
+          <t>K-A2</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>S-GIZMO</t>
+          <t>S-GADGET</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Gizmo A4</t>
+          <t>Gadget A2</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Gizmo</t>
+          <t>Gadget</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Gizmo A4 — single</t>
+          <t>Gadget A2 — single</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1567,20 +1567,20 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>iris@example.com</t>
+          <t>dave@example.com</t>
         </is>
       </c>
       <c r="L11" s="1" t="n">
-        <v>45762.5</v>
+        <v>45741.5</v>
       </c>
       <c r="M11" s="1" t="n">
-        <v>45762.83333333334</v>
+        <v>45741.83333333334</v>
       </c>
       <c r="N11" s="1" t="n">
-        <v>45765.5</v>
+        <v>45744.5</v>
       </c>
       <c r="O11" t="n">
-        <v>24</v>
+        <v>15.99</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
@@ -1588,16 +1588,16 @@
         </is>
       </c>
       <c r="Q11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>Indianapolis</t>
+          <t>Aurora</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>CO</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1607,16 +1607,1096 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>TRK-P4-O9</t>
+          <t>TRK-P4-A10</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>FedEx</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="W11" t="inlineStr"/>
       <c r="X11" t="inlineStr">
+        <is>
+          <t>FBA</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>p4:US</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>P4-B1</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>M-A5</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>K-A5</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>S-SPROCKET</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Sprocket A5</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Sprocket</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Sprocket A5 — single</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>alice@example.com</t>
+        </is>
+      </c>
+      <c r="L12" s="1" t="n">
+        <v>45720.5</v>
+      </c>
+      <c r="M12" s="1" t="n">
+        <v>45720.83333333334</v>
+      </c>
+      <c r="N12" s="1" t="n">
+        <v>45723.5</v>
+      </c>
+      <c r="O12" t="n">
+        <v>7.49</v>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q12" t="n">
+        <v>1</v>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Austin</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>TRK-P4-B1</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>FedEx</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr"/>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>FBA</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>p4:US</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>P4-B2</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>A6</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>M-A6</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>K-A6</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>S-BRACKET</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Bracket A6</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Bracket</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Bracket A6 — single</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>alice@example.com</t>
+        </is>
+      </c>
+      <c r="L13" s="1" t="n">
+        <v>45726.5</v>
+      </c>
+      <c r="M13" s="1" t="n">
+        <v>45726.83333333334</v>
+      </c>
+      <c r="N13" s="1" t="n">
+        <v>45729.5</v>
+      </c>
+      <c r="O13" t="n">
+        <v>12.25</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q13" t="n">
+        <v>1</v>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>TRK-P4-B2</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>FedEx</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr"/>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>FBA</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>p4:US</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>P4-B3</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>A7</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>M-A7</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>K-A7</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>S-LEVER</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Lever A7</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Lever</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Lever A7 — single</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>alice@example.com</t>
+        </is>
+      </c>
+      <c r="L14" s="1" t="n">
+        <v>45733.5</v>
+      </c>
+      <c r="M14" s="1" t="n">
+        <v>45733.83333333334</v>
+      </c>
+      <c r="N14" s="1" t="n">
+        <v>45736.5</v>
+      </c>
+      <c r="O14" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q14" t="n">
+        <v>1</v>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Dallas</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>TRK-P4-B3</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>FedEx</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr"/>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>FBA</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>p4:US</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>P4-B4</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>A8</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>M-A8</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>K-A8</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>S-PULLEY</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Pulley A8</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Pulley</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Pulley A8 — single</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>alice@example.com</t>
+        </is>
+      </c>
+      <c r="L15" s="1" t="n">
+        <v>45747.5</v>
+      </c>
+      <c r="M15" s="1" t="n">
+        <v>45747.83333333334</v>
+      </c>
+      <c r="N15" s="1" t="n">
+        <v>45750.5</v>
+      </c>
+      <c r="O15" t="n">
+        <v>26</v>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q15" t="n">
+        <v>1</v>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Plano</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>TRK-P4-B4</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>FedEx</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr"/>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>FBA</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>p4:US</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>P4-B5</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>M-A5</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>K-A5</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>S-SPROCKET</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Sprocket A5</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Sprocket</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Sprocket A5 — single</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>bob@example.com</t>
+        </is>
+      </c>
+      <c r="L16" s="1" t="n">
+        <v>45723.5</v>
+      </c>
+      <c r="M16" s="1" t="n">
+        <v>45723.83333333334</v>
+      </c>
+      <c r="N16" s="1" t="n">
+        <v>45726.5</v>
+      </c>
+      <c r="O16" t="n">
+        <v>7.49</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q16" t="n">
+        <v>1</v>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Boston</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>TRK-P4-B5</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>FedEx</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr"/>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>FBA</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>p4:US</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>P4-B6</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>A6</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>M-A6</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>K-A6</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>S-BRACKET</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Bracket A6</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Bracket</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Bracket A6 — single</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>bob@example.com</t>
+        </is>
+      </c>
+      <c r="L17" s="1" t="n">
+        <v>45736.5</v>
+      </c>
+      <c r="M17" s="1" t="n">
+        <v>45736.83333333334</v>
+      </c>
+      <c r="N17" s="1" t="n">
+        <v>45739.5</v>
+      </c>
+      <c r="O17" t="n">
+        <v>12.25</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q17" t="n">
+        <v>1</v>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Cambridge</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>TRK-P4-B6</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>FedEx</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr"/>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>FBA</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>p4:US</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>P4-B7</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>A7</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>M-A7</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>K-A7</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>S-LEVER</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Lever A7</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Lever</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Lever A7 — single</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>bob@example.com</t>
+        </is>
+      </c>
+      <c r="L18" s="1" t="n">
+        <v>45749.5</v>
+      </c>
+      <c r="M18" s="1" t="n">
+        <v>45749.83333333334</v>
+      </c>
+      <c r="N18" s="1" t="n">
+        <v>45752.5</v>
+      </c>
+      <c r="O18" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q18" t="n">
+        <v>1</v>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>Brookline</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>TRK-P4-B7</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>FedEx</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr"/>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>FBA</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>p4:US</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>P4-B8</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>M-A5</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>K-A5</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>S-SPROCKET</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Sprocket A5</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Sprocket</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Sprocket A5 — single</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>dave@example.com</t>
+        </is>
+      </c>
+      <c r="L19" s="1" t="n">
+        <v>45730.5</v>
+      </c>
+      <c r="M19" s="1" t="n">
+        <v>45730.83333333334</v>
+      </c>
+      <c r="N19" s="1" t="n">
+        <v>45733.5</v>
+      </c>
+      <c r="O19" t="n">
+        <v>7.49</v>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q19" t="n">
+        <v>1</v>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>Denver</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>TRK-P4-B8</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>FedEx</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr"/>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>FBA</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>p4:US</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>P4-B9</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>A6</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>M-A6</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>K-A6</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>S-BRACKET</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Bracket A6</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Bracket</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Bracket A6 — single</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>dave@example.com</t>
+        </is>
+      </c>
+      <c r="L20" s="1" t="n">
+        <v>45743.5</v>
+      </c>
+      <c r="M20" s="1" t="n">
+        <v>45743.83333333334</v>
+      </c>
+      <c r="N20" s="1" t="n">
+        <v>45746.5</v>
+      </c>
+      <c r="O20" t="n">
+        <v>12.25</v>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q20" t="n">
+        <v>1</v>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>Lakewood</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>TRK-P4-B9</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>FedEx</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr"/>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>FBA</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>p4:US</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>P4-B10</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>A7</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>M-A7</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>K-A7</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>S-LEVER</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Lever A7</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Lever</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Lever A7 — single</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>dave@example.com</t>
+        </is>
+      </c>
+      <c r="L21" s="1" t="n">
+        <v>45755.5</v>
+      </c>
+      <c r="M21" s="1" t="n">
+        <v>45755.83333333334</v>
+      </c>
+      <c r="N21" s="1" t="n">
+        <v>45758.5</v>
+      </c>
+      <c r="O21" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q21" t="n">
+        <v>1</v>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Aurora</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>TRK-P4-B10</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>FedEx</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr"/>
+      <c r="X21" t="inlineStr">
         <is>
           <t>FBA</t>
         </is>

</xml_diff>